<commit_message>
descasamento: inclui todas as fontes no custo sem receita
Custo sem receita sobe de R$39K para R$3.9M ao incluir
margem_pessoas e margem_projetos além de rac_pessoas.
126 PEPs com custo mas sem receita no MapaReceita.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/descasamento_receita_custo_q4.xlsx
+++ b/backend/descasamento_receita_custo_q4.xlsx
@@ -556,12 +556,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 39.816,84</t>
+          <t>R$ 3.900.373,50</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 pessoas</t>
+          <t>62 PEPs — rac_pessoas + margem_pessoas + margem_projetos</t>
         </is>
       </c>
     </row>
@@ -5457,7 +5457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5500,208 +5500,4645 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BR07</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BR07CLP00126.0.1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>BRCPF00671466780</t>
-        </is>
-      </c>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Adriana Fonseca Pinto</t>
+          <t>BANCO OURINVEST S/A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-483.93</v>
+        <v>-334557.049937007</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>R$ -483,93</t>
+          <t>R$ -334.557,05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BR07</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BR07CLP00126.0.1</t>
+          <t>BR02INP00304.1.1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BRCPF39496114873</t>
+          <t>BRCPF10658257811</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mariana Goto da Silva</t>
+          <t>ALESSANDRO PORRO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>316.6799999999998</v>
+        <v>-228355.76</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>R$ 316,68</t>
+          <t>R$ -228.355,76</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BR02</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BR02CLP000123.0.1</t>
+          <t>BR02INP00018.1.1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BRCPF23633749837</t>
+          <t>BRCPF30095686819</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EVELYN HIKARI YOSHITANI</t>
+          <t>Alberto Yamamoto</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>727.05</v>
+        <v>-186000</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>R$ 727,05</t>
+          <t>R$ -186.000,00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BR02</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BR02CLP000312.0.1</t>
+          <t>BR02BU2007.1.1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BRCPF09728873697</t>
+          <t>BRCPF30645911852</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CATHARINA  GAISSLER SANTOS</t>
+          <t>Fernando Artea</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1378.38</v>
+        <v>-142500</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>R$ 1.378,38</t>
+          <t>R$ -142.500,00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BR02</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BR02CLP000234.0.1</t>
+          <t>BR02BU2014.1.1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BRCPF43991981840</t>
+          <t>BRCPF39634273882</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Patricia Costa Fernandes</t>
+          <t>Rafael Rosa</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4319.14</v>
+        <v>-141900</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>R$ 4.319,14</t>
+          <t>R$ -141.900,00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BR02BU2009.1.1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BRCPF24653329885</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Alexsandro Monteiro</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>-135000</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>R$ -135.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BR02INP00012.1.1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BRCPF39314129896</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Vinicius Galera</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>-129999.99</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>R$ -129.999,99</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BR02INP0001.1.1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BRCPF32789724814</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rodrigo Santos</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>-101713.74</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>R$ -101.713,74</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BR02BU2008.1.1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BRCPF10412494620</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Henrique Carneiro</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>-93845.58</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>R$ -93.845,58</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BR02BU2013.1.1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BRCPF38911757870</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Marcelo Mazini</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>-93000</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>R$ -93.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BR02INP00003.1.1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BRCPF32207787800</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Eric Vieira</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>-82500</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>R$ -82.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BR02BU2005.1.1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BRCPF19071224864</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ricardo Henrique</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>-78000</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>R$ -78.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BRCPF07223083883</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Helen Passos</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>-73617.07000000001</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>R$ -73.617,07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BR02BU2005.1.1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BRCPF35322478876</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Daniel Machado</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>-73500</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>R$ -73.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BR02INP00011.1.1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BRCPF30497828898</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Roberto Caracciolo</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>-72000</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>R$ -72.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BR02CLP00115.1.1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BRCPF33657714847</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FERNANDO LISBOA</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>-72000</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>R$ -72.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BR02INP00037.1.1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BRCPF46138189825</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Felipe Correia</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>-66000</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>R$ -66.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BR02BO0304.1.1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BRCPF00261952080</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Leomar Junior</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>-66000</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>R$ -66.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BR02BU2008.1.1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BRCPF85409006615</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Danilo Macieira</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>-63000</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>R$ -63.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BRCPF17599284702</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>WILLIAN RODRIGUES</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>-62640</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>R$ -62.640,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BRCPF04095347902</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>John Silva</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>-62126.195</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>R$ -62.126,19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BR02BU2008.1.1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BRCPF06382222658</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Jamil Costa</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>-59150</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>R$ -59.150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BR02BU2006.1.1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BRCPF07597558929</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Luiz Nunes</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>-55536.405</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>R$ -55.536,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BR02BU2009.1.1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BRCPF14332209893</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>LEANDRO BRITO</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>-51652.8</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>R$ -51.652,80</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BRCPF09500671999</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Rodolfo Duarte</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>-48000</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>R$ -48.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BR02INP00003.1.2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BRCPF05918147730</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Fernando Goes</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>-47946.91</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>R$ -47.946,91</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BR02BU2015.1.1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BRCPF31584847816</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Kattia Cerri</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>-45000</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>R$ -45.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BR02BO0303.1.2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BRCPF03943840670</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Thiago Azevedo</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>-42000</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>R$ -42.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BR02BO0303.1.1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BRCPF03943840670</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Thiago Azevedo</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>-42000</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>R$ -42.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BR02BU0007.1.1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BRCPF48679899836</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Nathan Lima</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>-40500</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>R$ -40.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BRCPF04095347902</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>John Silva</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>-39876.195</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>R$ -39.876,19</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BR02BU2020.1.1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BRCPF09323849944</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Willian Santos</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>-38643.65</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>R$ -38.643,65</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BR02BU2020.1.1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BRCPF07976443429</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>LYSSA BACKSCHAT</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>-36000</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>R$ -36.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BRCPF03008249710</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pedro Neto</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>-35700</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>R$ -35.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BR02INP00006.1.3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BRCPF21248980867</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Samantha Garcia</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>-30453.5</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>R$ -30.453,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BRCPF06333426962</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Luiz Marin</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>R$ -30.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BR02BU2020.1.1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BRCPF23012910816-1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Thiago Sousa</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>-24968.12526166534</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>R$ -24.968,13</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>BR02BU2015.1.1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BRCPF01106346750</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Juliana Veronese</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>-24000</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>R$ -24.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BR02INP00004.1.1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BRCPF01106346750</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Juliana Veronese</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>-24000</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>R$ -24.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BRCPF43173761804</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Aldrei Mecias Mirandą</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>-22842.19650967741</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>R$ -22.842,20</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BR02BU2012.1.1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BRCPF46632834892</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Gabriel Sanzone</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>-22420.64</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>R$ -22.420,64</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BR02CLP000412.1.1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BRCPF46632834892</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Gabriel Sanzone</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>-22420.64</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>R$ -22.420,64</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BRCPF02853967220</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Lennon Roberto Almeida Ribeiro</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>-22273.75307610692</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>R$ -22.273,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BR07CLP00102.1.1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BRCPF37001274801</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Tiago Lee</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>-19430.95567805194</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>R$ -19.430,96</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BR02BO0302.1.2</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BRCPF01526924013</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>LEONARDO DORNELLES</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>-19200</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>R$ -19.200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BRCPF44299499808</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Eder Rebernisek Mariano</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>-19064.20301115029</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>R$ -19.064,20</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BRCPF37832008814</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Geison Cardoso de Lima</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>-18987.02</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>R$ -18.987,02</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BR02BU2009.1.1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>BRCPF38160828829</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Bruno Sousa</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>-18900</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>R$ -18.900,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BR02BU2009.1.1</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BRCPF05148962801</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ROGERIO SEGALA</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>-17772.48</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>R$ -17.772,48</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>BRCPF45892862895</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Matheus Castro Ciuffi</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>-17748.03326383431</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>R$ -17.748,03</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>BRCPF44024982877</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>VinIcius Arantes Paiva</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>-17203.87469368891</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>R$ -17.203,87</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>BRCPF07622790877</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Ulysses Maria Samenho Junior</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>-16800</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>R$ -16.800,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>BR02BU2010.1.1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>BRCPF32207787800</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Eric Vieira</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>-16500</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>R$ -16.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BRCPF35416128860</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>DENISE  DOS SANTOS CAMPANHA</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>-15360.95685859201</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>R$ -15.360,96</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>BRCPF70048033413</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Judson Kerller Alves Morais Junior</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>-15130.27708751075</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>R$ -15.130,28</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>BRCPF39255632884</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Matheus Akira Mimura</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>-14812.50098343426</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>R$ -14.812,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>BRCPF39320012814</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Gabriel Rodrigues Ramos de Oliveira</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>-14500</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>R$ -14.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BRCPF44605930841</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Matheus Batista Correa</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>-13708.9685465369</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>R$ -13.708,97</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BRCPF44753720896</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Victor Mota Gonçalves</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>-13451.09315796554</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>R$ -13.451,09</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>BRCPF05167424771</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>FERNANDO NETO</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>-13347.5</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>R$ -13.347,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>BR02CLP00031.1.1</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>BRCPF05167424771</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>FERNANDO NETO</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>-13347.5</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>R$ -13.347,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>BRCPF52324634899</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Henrique Cesar de Souza</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>-13255.83110613576</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>R$ -13.255,83</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>BRCPF49210208846</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Gustavo Rodrigues da Silva</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>-13207.27436894465</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>R$ -13.207,27</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>BR02CLP00241.1.1</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>BRCPF38133115892</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Thiago Giraldes</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>-13203.508</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>R$ -13.203,51</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>BR02CLP000115.1.1</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>BRCPF38133115892</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Thiago Giraldes</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>-13203.508</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>R$ -13.203,51</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BR02INP000013.1.1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>BRCPF21248980867</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Samantha Garcia</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-12</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>-13051.5</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>R$ -13.051,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>BRCPF46884961848</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jonata Willian Pereira da Silva </t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>-12944.65600266752</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>R$ -12.944,66</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>BRCPF43387015879</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gilson da Silva Fonseca </t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>-12916.52640100733</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>R$ -12.916,53</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BR07CLP00102.1.1</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>BRCPF05008651161</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Guilherme Laudensack</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>-12817.17085527272</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>R$ -12.817,17</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>BRCPF40460038800</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Augusto Cesar dos Anjos Santana</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>-12703.22011891936</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>R$ -12.703,22</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>BRCPF08483209640</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Marcos Paulo do Nascimento</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>-12032.52049387173</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>R$ -12.032,52</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>BR02CLP00241.1.1</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>BRCPF06382222658</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Jamil Costa</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>-11830</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>R$ -11.830,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>BRCPF48830260860</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Yury Ryan Nascimento Godinho</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>-11142.82104342082</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>R$ -11.142,82</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>BRCPF43042433811</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Renan Guilherme de Sousa</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>-11035.04</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>R$ -11.035,04</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>BR02CLP00178.1.1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>BRCPF96792469653</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Claudecir Silva</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>-10920</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>R$ -10.920,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BR02INP000013.1.1</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>BRCPF04182369688</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Manuela Antunes</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>-10483</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>R$ -10.483,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BR02INP000010.1.1</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>BRCPF04182369688</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Manuela Antunes</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>-10483</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>R$ -10.483,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BR02INP000015.1.1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>BRCPF04182369688</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Manuela Antunes</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>-10483</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>R$ -10.483,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>BR07CLP00165.1.1</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>BRCPF37672117858</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Samuel Valim</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>-10359.77239494949</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>R$ -10.359,77</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>BR07CLP00102.1.3</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>BRCPF37001274801</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Tiago Lee</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>-10050.49431623376</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>R$ -10.050,49</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>BR02CLP000300.1.1</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>DISTRITO TECNOLOGIA E SERVICOS S.A.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>R$ -10.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BR02CLP000300.1.1</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>BRCPF44746363846</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Murilo Bagodi</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>R$ -10.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>BRCPF46975818819</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>YURI  FERNANDES DA SILVA</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>-9618.203213542518</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>R$ -9.618,20</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BR02CLP000815.1.1</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>BRCPF38544223850</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Rafaella Costa</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>-9585.5</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>R$ -9.585,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>BR02INP00004.1.1</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>BRCPF38544223850</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Rafaella Costa</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>-9585.5</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>R$ -9.585,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>BR02BU2010.1.1</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>BRCPF05918147730</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Fernando Goes</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>-9000</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>R$ -9.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>BR07CLP00180.1.27</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>BRCPF70769399169</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>AUGUSTO SAVI</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>-8818.816477155684</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>R$ -8.818,82</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>BR02CLP000513.1.1</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>BRCPF70605475172</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>RAPHAEL REIS</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>-8400</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>R$ -8.400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>BR02INP000017.1.1</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>BRCPF29823044813</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Maria Gomes</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>-8232.5</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>R$ -8.232,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>BR02INP000013.1.1</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BRCPF09728873697</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>CATHARINA SANTOS</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>-8228.333333333332</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>R$ -8.228,33</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BR02INP000021.1.1</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>BRCPF09728873697</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>CATHARINA SANTOS</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>-8228.333333333332</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>R$ -8.228,33</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BR02INP000013.1.1</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BRCPF32503272800</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Murilo Souza</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>R$ -8.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BR02CLP00161.1.1</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>BRCPF32503272800</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Murilo Souza</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>R$ -8.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BR02INP00002.1.2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>BRCPF07969644910</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Luiz Kekis</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>-7694.6</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>R$ -7.694,60</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>BRCPF01321990685</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Carlos Souza</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>-7326.25</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>R$ -7.326,25</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>BR02CLP00178.1.1</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BRCPF03008249710</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Pedro Neto</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>-7140</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>R$ -7.140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>BR02INP00004.1.1</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>BRCPF39305416888</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Marcelo Reis</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>-6526.1</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>R$ -6.526,10</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>BR02CLP00031.1.1</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>BRCPF84585447687</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Silvio Jose de Souza</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>-5830</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>R$ -5.830,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>BRCPF09396903906</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Ronaldo Bruno De Souza Santos</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>-5826.666666666666</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>R$ -5.826,67</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BR02CLP00091.1.1</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>BRCPF36103714800</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Rodrigo Santos</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>-5681.386666666666</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>R$ -5.681,39</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>BR02INP00004.1.1</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BRCPF43991981840</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Patricia Fernandes</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>-5075</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>R$ -5.075,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>BR02INP00004.1.2</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BRCPF43991981840</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Patricia Fernandes</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>-5075</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>R$ -5.075,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>BRCPF06908239918</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Ricardo Lopes</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>-5060</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>R$ -5.060,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BRCPF05779922608</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Danilo Dumba</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>-4968.425</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>R$ -4.968,43</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BR02CLP000809.1.1</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>BRCPF36995162889</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Diego Fernandes</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>-4830.755</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>R$ -4.830,76</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BR02INP000010.1.1</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BRCPF21248980867</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Samantha Garcia</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>-4350.5</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>R$ -4.350,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BR02INP000015.1.1</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>BRCPF21248980867</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Samantha Garcia</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>-4350.5</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>R$ -4.350,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>BR07CLP00102.1.5</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BRCPF05008651161</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Guilherme Laudensack</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>-4272.390285090907</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>R$ -4.272,39</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>BRCPF38133115892</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Thiago Giraldes</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>-3963.508</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>R$ -3.963,51</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>BR07CLP00015.0.1</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BRCPF40861701836</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>THIAGO RIBEIRO RETAMIRO</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>-3818.08</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>R$ -3.818,08</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BRCPF00080118003</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Fabio Winck</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>-3800.08125</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>R$ -3.800,08</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>BR02BU2020.1.1</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>BRCPF43642053890</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>MATEUS OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>-3420</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>R$ -3.420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>BR02CLP000819.1.1</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>BRCPF43642053890</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>MATEUS OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>-3420</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>R$ -3.420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>BRCPF84585447687</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Silvio Jose de Souza</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>-3410</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>R$ -3.410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>BR02INP000011.1.1</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>BRCPF29823044813</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Maria Gomes</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>-3293</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>R$ -3.293,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>BR02INP000012.1.1</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>BRCPF29823044813</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Maria Gomes</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>-3293</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>R$ -3.293,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>BR02INP00004.1.1</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>BRCPF29823044813</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Maria Gomes</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>-3293</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>R$ -3.293,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>BR02INP000013.1.1</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>BRCPF29823044813</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Maria Gomes</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2025-11, 2025-12</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>-3293</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>R$ -3.293,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>BR02CLP000115.1.1</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>BRCPF01321990685</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Carlos Souza</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>-3006.25</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>R$ -3.006,25</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>BR07CLP00102.1.1</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>BRCPF33656123861</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Diego Grigorjevs</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-12</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>-2924.811818961039</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>R$ -2.924,81</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>BR07CLP00165.1.1</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>BRCPF41904875890-1</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>EMILY IZABELLE GONCALVES</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>-2779.144924</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>R$ -2.779,14</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>BR02INP00002.1.2</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>BRCPF33617629873</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Danielle Peraccini</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-12</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>-2700</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>R$ -2.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>BR02CLP00241.1.1</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>BRCPF11340898640</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Matheus Fraga</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>-2300</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>R$ -2.300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>BRCPF11340898640</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Matheus Fraga</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>-2300</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>R$ -2.300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>FCamara</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>BR02INP00009.1.1</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>BRCPF48959910678</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Joao Braccini</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2025-10, 2025-11</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>-1635.555555555555</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>R$ -1.635,56</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>BR07CLP00180.1.4</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>BRCPF40625247833</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Luana Arena</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>-1442.829992181818</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>R$ -1.442,83</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Hyper</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>BR07CLP00102.1.5</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>BRCPF33656123861</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Diego Grigorjevs</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>-1364.912182181818</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>R$ -1.364,91</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>BR07</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>BR07CLP00126.0.1</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>BRCPF00671466780</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Adriana Fonseca Pinto</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>-483.93</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>R$ -483,93</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>BR07</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>BR07CLP00126.0.1</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>BRCPF39496114873</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Mariana Goto da Silva</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>316.6799999999998</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>R$ 316,68</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
           <t>BR02</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>BR02CLP000123.0.1</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>BRCPF23633749837</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>EVELYN HIKARI YOSHITANI</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>727.05</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>R$ 727,05</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>BR02</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>BR02CLP000312.0.1</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>BRCPF09728873697</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>CATHARINA  GAISSLER SANTOS</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>1378.38</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>R$ 1.378,38</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>BR02</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BR02CLP000234.0.1</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>BRCPF43991981840</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Patricia Costa Fernandes</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>4319.14</v>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>R$ 4.319,14</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>BR02</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
         <is>
           <t>BR02CLP00115.0.1</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>BRCPF40254370829</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D134" t="inlineStr">
         <is>
           <t>Guilherme Manucci</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E134" t="inlineStr">
         <is>
           <t>2025-10, 2025-11</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F134" t="n">
         <v>33559.52</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G134" t="inlineStr">
         <is>
           <t>R$ 33.559,52</t>
         </is>

</xml_diff>

<commit_message>
fix: usa nome completo do AE em todos os filtros de budget e lb_trigger
O filtro de budget_receita e lb_trigger usava nome_n (nome parcial de busca)
em vez do nome completo normalizado da pessoa, deixando clientes_detalhe
vazio e trigger_lb em 0 quando chamado com nome abreviado via API.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/descasamento_receita_custo_q4.xlsx
+++ b/backend/descasamento_receita_custo_q4.xlsx
@@ -556,12 +556,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 3.900.373,50</t>
+          <t>R$ 3.923.623,85</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>62 PEPs — rac_pessoas + margem_pessoas + margem_projetos</t>
+          <t>68 PEPs — rac_pessoas + margem_pessoas + margem_projetos</t>
         </is>
       </c>
     </row>
@@ -5457,7 +5457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6756,35 +6756,31 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>BR08</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BR02BU2020.1.1</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>BRCPF23012910816-1</t>
-        </is>
-      </c>
+          <t>BR08CLP00012.0.1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Thiago Sousa</t>
+          <t>Kewin Sachtleben</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11, 2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>-24968.12526166534</v>
+        <v>-27548.02</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>R$ -24.968,13</t>
+          <t>R$ -27.548,02</t>
         </is>
       </c>
     </row>
@@ -6796,30 +6792,30 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BR02BU2015.1.1</t>
+          <t>BR02BU2020.1.1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>BRCPF01106346750</t>
+          <t>BRCPF23012910816-1</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Juliana Veronese</t>
+          <t>Thiago Sousa</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>-24000</v>
+        <v>-24968.12526166534</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>R$ -24.000,00</t>
+          <t>R$ -24.968,13</t>
         </is>
       </c>
     </row>
@@ -6831,7 +6827,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BR02INP00004.1.1</t>
+          <t>BR02BU2015.1.1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6846,7 +6842,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-10, 2025-11</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -6866,30 +6862,30 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02INP00004.1.1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BRCPF43173761804</t>
+          <t>BRCPF01106346750</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Aldrei Mecias Mirandą</t>
+          <t>Juliana Veronese</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>-22842.19650967741</v>
+        <v>-24000</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>R$ -22.842,20</t>
+          <t>R$ -24.000,00</t>
         </is>
       </c>
     </row>
@@ -6901,30 +6897,30 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BR02BU2012.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>BRCPF46632834892</t>
+          <t>BRCPF43173761804</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Gabriel Sanzone</t>
+          <t>Aldrei Mecias Mirandą</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>-22420.64</v>
+        <v>-22842.19650967741</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>R$ -22.420,64</t>
+          <t>R$ -22.842,20</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6932,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BR02CLP000412.1.1</t>
+          <t>BR02BU2012.1.1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6971,100 +6967,100 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02CLP000412.1.1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>BRCPF02853967220</t>
+          <t>BRCPF46632834892</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Lennon Roberto Almeida Ribeiro</t>
+          <t>Gabriel Sanzone</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-11</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>-22273.75307610692</v>
+        <v>-22420.64</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>R$ -22.273,75</t>
+          <t>R$ -22.420,64</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BR07CLP00102.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BRCPF37001274801</t>
+          <t>BRCPF02853967220</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Tiago Lee</t>
+          <t>Lennon Roberto Almeida Ribeiro</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>-19430.95567805194</v>
+        <v>-22273.75307610692</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>R$ -19.430,96</t>
+          <t>R$ -22.273,75</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BR02BO0302.1.2</t>
+          <t>BR07CLP00102.1.1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BRCPF01526924013</t>
+          <t>BRCPF37001274801</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>LEONARDO DORNELLES</t>
+          <t>Tiago Lee</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>-19200</v>
+        <v>-19430.95567805194</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>R$ -19.200,00</t>
+          <t>R$ -19.430,96</t>
         </is>
       </c>
     </row>
@@ -7076,17 +7072,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02BO0302.1.2</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BRCPF44299499808</t>
+          <t>BRCPF01526924013</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Eder Rebernisek Mariano</t>
+          <t>LEONARDO DORNELLES</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -7095,11 +7091,11 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>-19064.20301115029</v>
+        <v>-19200</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>R$ -19.064,20</t>
+          <t>R$ -19.200,00</t>
         </is>
       </c>
     </row>
@@ -7116,12 +7112,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BRCPF37832008814</t>
+          <t>BRCPF44299499808</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Geison Cardoso de Lima</t>
+          <t>Eder Rebernisek Mariano</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -7130,11 +7126,11 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>-18987.02</v>
+        <v>-19064.20301115029</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>R$ -18.987,02</t>
+          <t>R$ -19.064,20</t>
         </is>
       </c>
     </row>
@@ -7146,30 +7142,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BR02BU2009.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BRCPF38160828829</t>
+          <t>BRCPF37832008814</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Bruno Sousa</t>
+          <t>Geison Cardoso de Lima</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>-18900</v>
+        <v>-18987.02</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>R$ -18.900,00</t>
+          <t>R$ -18.987,02</t>
         </is>
       </c>
     </row>
@@ -7186,25 +7182,25 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BRCPF05148962801</t>
+          <t>BRCPF38160828829</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ROGERIO SEGALA</t>
+          <t>Bruno Sousa</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>-17772.48</v>
+        <v>-18900</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>R$ -17.772,48</t>
+          <t>R$ -18.900,00</t>
         </is>
       </c>
     </row>
@@ -7216,17 +7212,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02BU2009.1.1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>BRCPF45892862895</t>
+          <t>BRCPF05148962801</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Matheus Castro Ciuffi</t>
+          <t>ROGERIO SEGALA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -7235,11 +7231,11 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>-17748.03326383431</v>
+        <v>-17772.48</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>R$ -17.748,03</t>
+          <t>R$ -17.772,48</t>
         </is>
       </c>
     </row>
@@ -7256,12 +7252,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>BRCPF44024982877</t>
+          <t>BRCPF45892862895</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>VinIcius Arantes Paiva</t>
+          <t>Matheus Castro Ciuffi</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -7270,11 +7266,11 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>-17203.87469368891</v>
+        <v>-17748.03326383431</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>R$ -17.203,87</t>
+          <t>R$ -17.748,03</t>
         </is>
       </c>
     </row>
@@ -7291,12 +7287,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>BRCPF07622790877</t>
+          <t>BRCPF44024982877</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ulysses Maria Samenho Junior</t>
+          <t>VinIcius Arantes Paiva</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -7305,11 +7301,11 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>-16800</v>
+        <v>-17203.87469368891</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>R$ -16.800,00</t>
+          <t>R$ -17.203,87</t>
         </is>
       </c>
     </row>
@@ -7321,30 +7317,30 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>BR02BU2010.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BRCPF32207787800</t>
+          <t>BRCPF07622790877</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Eric Vieira</t>
+          <t>Ulysses Maria Samenho Junior</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>-16500</v>
+        <v>-16800</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>R$ -16.500,00</t>
+          <t>R$ -16.800,00</t>
         </is>
       </c>
     </row>
@@ -7356,30 +7352,30 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02BU2010.1.1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BRCPF35416128860</t>
+          <t>BRCPF32207787800</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DENISE  DOS SANTOS CAMPANHA</t>
+          <t>Eric Vieira</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>-15360.95685859201</v>
+        <v>-16500</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>R$ -15.360,96</t>
+          <t>R$ -16.500,00</t>
         </is>
       </c>
     </row>
@@ -7396,12 +7392,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>BRCPF70048033413</t>
+          <t>BRCPF35416128860</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Judson Kerller Alves Morais Junior</t>
+          <t>DENISE  DOS SANTOS CAMPANHA</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -7410,11 +7406,11 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>-15130.27708751075</v>
+        <v>-15360.95685859201</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>R$ -15.130,28</t>
+          <t>R$ -15.360,96</t>
         </is>
       </c>
     </row>
@@ -7431,12 +7427,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>BRCPF39255632884</t>
+          <t>BRCPF70048033413</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Matheus Akira Mimura</t>
+          <t>Judson Kerller Alves Morais Junior</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -7445,11 +7441,11 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>-14812.50098343426</v>
+        <v>-15130.27708751075</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>R$ -14.812,50</t>
+          <t>R$ -15.130,28</t>
         </is>
       </c>
     </row>
@@ -7466,12 +7462,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>BRCPF39320012814</t>
+          <t>BRCPF39255632884</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Gabriel Rodrigues Ramos de Oliveira</t>
+          <t>Matheus Akira Mimura</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -7480,11 +7476,11 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>-14500</v>
+        <v>-14812.50098343426</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>R$ -14.500,00</t>
+          <t>R$ -14.812,50</t>
         </is>
       </c>
     </row>
@@ -7501,12 +7497,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>BRCPF44605930841</t>
+          <t>BRCPF39320012814</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Matheus Batista Correa</t>
+          <t>Gabriel Rodrigues Ramos de Oliveira</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -7515,11 +7511,11 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>-13708.9685465369</v>
+        <v>-14500</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>R$ -13.708,97</t>
+          <t>R$ -14.500,00</t>
         </is>
       </c>
     </row>
@@ -7536,12 +7532,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BRCPF44753720896</t>
+          <t>BRCPF44605930841</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Victor Mota Gonçalves</t>
+          <t>Matheus Batista Correa</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -7550,11 +7546,11 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>-13451.09315796554</v>
+        <v>-13708.9685465369</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>R$ -13.451,09</t>
+          <t>R$ -13.708,97</t>
         </is>
       </c>
     </row>
@@ -7566,30 +7562,30 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BRCPF05167424771</t>
+          <t>BRCPF44753720896</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>FERNANDO NETO</t>
+          <t>Victor Mota Gonçalves</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>-13347.5</v>
+        <v>-13451.09315796554</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>R$ -13.347,50</t>
+          <t>R$ -13.451,09</t>
         </is>
       </c>
     </row>
@@ -7636,30 +7632,30 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BRCPF52324634899</t>
+          <t>BRCPF05167424771</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Henrique Cesar de Souza</t>
+          <t>FERNANDO NETO</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>-13255.83110613576</v>
+        <v>-13347.5</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>R$ -13.255,83</t>
+          <t>R$ -13.347,50</t>
         </is>
       </c>
     </row>
@@ -7676,12 +7672,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>BRCPF49210208846</t>
+          <t>BRCPF52324634899</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Gustavo Rodrigues da Silva</t>
+          <t>Henrique Cesar de Souza</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -7690,11 +7686,11 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>-13207.27436894465</v>
+        <v>-13255.83110613576</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>R$ -13.207,27</t>
+          <t>R$ -13.255,83</t>
         </is>
       </c>
     </row>
@@ -7706,30 +7702,30 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>BR02CLP00241.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BRCPF38133115892</t>
+          <t>BRCPF49210208846</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Thiago Giraldes</t>
+          <t>Gustavo Rodrigues da Silva</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>-13203.508</v>
+        <v>-13207.27436894465</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>R$ -13.203,51</t>
+          <t>R$ -13.207,27</t>
         </is>
       </c>
     </row>
@@ -7776,30 +7772,30 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BR02INP000013.1.1</t>
+          <t>BR02CLP00241.1.1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>BRCPF21248980867</t>
+          <t>BRCPF38133115892</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Samantha Garcia</t>
+          <t>Thiago Giraldes</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025-10, 2025-12</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>-13051.5</v>
+        <v>-13203.508</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>R$ -13.051,50</t>
+          <t>R$ -13.203,51</t>
         </is>
       </c>
     </row>
@@ -7811,30 +7807,30 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02INP000013.1.1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>BRCPF46884961848</t>
+          <t>BRCPF21248980867</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jonata Willian Pereira da Silva </t>
+          <t>Samantha Garcia</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-12</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>-12944.65600266752</v>
+        <v>-13051.5</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>R$ -12.944,66</t>
+          <t>R$ -13.051,50</t>
         </is>
       </c>
     </row>
@@ -7851,12 +7847,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>BRCPF43387015879</t>
+          <t>BRCPF46884961848</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gilson da Silva Fonseca </t>
+          <t xml:space="preserve">Jonata Willian Pereira da Silva </t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -7865,81 +7861,81 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>-12916.52640100733</v>
+        <v>-12944.65600266752</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>R$ -12.916,53</t>
+          <t>R$ -12.944,66</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>BR07CLP00102.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>BRCPF05008651161</t>
+          <t>BRCPF43387015879</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Guilherme Laudensack</t>
+          <t xml:space="preserve">Gilson da Silva Fonseca </t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>-12817.17085527272</v>
+        <v>-12916.52640100733</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>R$ -12.817,17</t>
+          <t>R$ -12.916,53</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR07CLP00102.1.1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>BRCPF40460038800</t>
+          <t>BRCPF05008651161</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Augusto Cesar dos Anjos Santana</t>
+          <t>Guilherme Laudensack</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>-12703.22011891936</v>
+        <v>-12817.17085527272</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>R$ -12.703,22</t>
+          <t>R$ -12.817,17</t>
         </is>
       </c>
     </row>
@@ -7956,12 +7952,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>BRCPF08483209640</t>
+          <t>BRCPF40460038800</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Marcos Paulo do Nascimento</t>
+          <t>Augusto Cesar dos Anjos Santana</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -7970,11 +7966,11 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>-12032.52049387173</v>
+        <v>-12703.22011891936</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>R$ -12.032,52</t>
+          <t>R$ -12.703,22</t>
         </is>
       </c>
     </row>
@@ -7986,30 +7982,30 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>BR02CLP00241.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>BRCPF06382222658</t>
+          <t>BRCPF08483209640</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Jamil Costa</t>
+          <t>Marcos Paulo do Nascimento</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>-11830</v>
+        <v>-12032.52049387173</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>R$ -11.830,00</t>
+          <t>R$ -12.032,52</t>
         </is>
       </c>
     </row>
@@ -8021,30 +8017,30 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02CLP00241.1.1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BRCPF48830260860</t>
+          <t>BRCPF06382222658</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Yury Ryan Nascimento Godinho</t>
+          <t>Jamil Costa</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>-11142.82104342082</v>
+        <v>-11830</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>R$ -11.142,82</t>
+          <t>R$ -11.830,00</t>
         </is>
       </c>
     </row>
@@ -8061,12 +8057,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>BRCPF43042433811</t>
+          <t>BRCPF48830260860</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Renan Guilherme de Sousa</t>
+          <t>Yury Ryan Nascimento Godinho</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -8075,11 +8071,11 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>-11035.04</v>
+        <v>-11142.82104342082</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>R$ -11.035,04</t>
+          <t>R$ -11.142,82</t>
         </is>
       </c>
     </row>
@@ -8091,17 +8087,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>BR02CLP00178.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>BRCPF96792469653</t>
+          <t>BRCPF43042433811</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Claudecir Silva</t>
+          <t>Renan Guilherme de Sousa</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -8110,11 +8106,11 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>-10920</v>
+        <v>-11035.04</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>R$ -10.920,00</t>
+          <t>R$ -11.035,04</t>
         </is>
       </c>
     </row>
@@ -8126,30 +8122,30 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>BR02INP000013.1.1</t>
+          <t>BR02CLP00178.1.1</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>BRCPF04182369688</t>
+          <t>BRCPF96792469653</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Manuela Antunes</t>
+          <t>Claudecir Silva</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>-10483</v>
+        <v>-10920</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>R$ -10.483,00</t>
+          <t>R$ -10.920,00</t>
         </is>
       </c>
     </row>
@@ -8161,7 +8157,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>BR02INP000010.1.1</t>
+          <t>BR02INP000015.1.1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -8196,7 +8192,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BR02INP000015.1.1</t>
+          <t>BR02INP000013.1.1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -8226,35 +8222,35 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>BR07CLP00165.1.1</t>
+          <t>BR02INP000010.1.1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>BRCPF37672117858</t>
+          <t>BRCPF04182369688</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Samuel Valim</t>
+          <t>Manuela Antunes</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>-10359.77239494949</v>
+        <v>-10483</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>R$ -10.359,77</t>
+          <t>R$ -10.483,00</t>
         </is>
       </c>
     </row>
@@ -8266,61 +8262,65 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>BR07CLP00102.1.3</t>
+          <t>BR07CLP00165.1.1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>BRCPF37001274801</t>
+          <t>BRCPF37672117858</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Tiago Lee</t>
+          <t>Samuel Valim</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>-10050.49431623376</v>
+        <v>-10359.77239494949</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>R$ -10.050,49</t>
+          <t>R$ -10.359,77</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>BR02CLP000300.1.1</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr"/>
+          <t>BR07CLP00102.1.3</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>BRCPF37001274801</t>
+        </is>
+      </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>DISTRITO TECNOLOGIA E SERVICOS S.A.</t>
+          <t>Tiago Lee</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>-10000</v>
+        <v>-10050.49431623376</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>R$ -10.000,00</t>
+          <t>R$ -10.050,49</t>
         </is>
       </c>
     </row>
@@ -8367,17 +8367,13 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>BRCPF46975818819</t>
-        </is>
-      </c>
+          <t>BR02CLP000300.1.1</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>YURI  FERNANDES DA SILVA</t>
+          <t>DISTRITO TECNOLOGIA E SERVICOS S.A.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -8386,11 +8382,11 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>-9618.203213542518</v>
+        <v>-10000</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>R$ -9.618,20</t>
+          <t>R$ -10.000,00</t>
         </is>
       </c>
     </row>
@@ -8402,17 +8398,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BR02CLP000815.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>BRCPF38544223850</t>
+          <t>BRCPF46975818819</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Rafaella Costa</t>
+          <t>YURI  FERNANDES DA SILVA</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -8421,11 +8417,11 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>-9585.5</v>
+        <v>-9618.203213542518</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>R$ -9.585,50</t>
+          <t>R$ -9.618,20</t>
         </is>
       </c>
     </row>
@@ -8437,7 +8433,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>BR02INP00004.1.1</t>
+          <t>BR02CLP000815.1.1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -8452,7 +8448,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -8472,52 +8468,52 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BR02BU2010.1.1</t>
+          <t>BR02INP00004.1.1</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>BRCPF05918147730</t>
+          <t>BRCPF38544223850</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Fernando Goes</t>
+          <t>Rafaella Costa</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>-9000</v>
+        <v>-9585.5</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>R$ -9.000,00</t>
+          <t>R$ -9.585,50</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>BR07CLP00180.1.27</t>
+          <t>BR02BU2010.1.1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>BRCPF70769399169</t>
+          <t>BRCPF05918147730</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>AUGUSTO SAVI</t>
+          <t>Fernando Goes</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -8526,33 +8522,33 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>-8818.816477155684</v>
+        <v>-9000</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>R$ -8.818,82</t>
+          <t>R$ -9.000,00</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>BR02CLP000513.1.1</t>
+          <t>BR07CLP00180.1.27</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>BRCPF70605475172</t>
+          <t>BRCPF70769399169</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>RAPHAEL REIS</t>
+          <t>AUGUSTO SAVI</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -8561,11 +8557,11 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>-8400</v>
+        <v>-8818.816477155684</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>R$ -8.400,00</t>
+          <t>R$ -8.818,82</t>
         </is>
       </c>
     </row>
@@ -8577,30 +8573,30 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>BR02INP000017.1.1</t>
+          <t>BR02CLP000513.1.1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>BRCPF29823044813</t>
+          <t>BRCPF70605475172</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Maria Gomes</t>
+          <t>RAPHAEL REIS</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>-8232.5</v>
+        <v>-8400</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>R$ -8.232,50</t>
+          <t>R$ -8.400,00</t>
         </is>
       </c>
     </row>
@@ -8612,30 +8608,30 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>BR02INP000013.1.1</t>
+          <t>BR02INP000017.1.1</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>BRCPF09728873697</t>
+          <t>BRCPF29823044813</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>CATHARINA SANTOS</t>
+          <t>Maria Gomes</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11, 2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>-8228.333333333332</v>
+        <v>-8232.5</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>R$ -8.228,33</t>
+          <t>R$ -8.232,50</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8643,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>BR02INP000021.1.1</t>
+          <t>BR02INP000013.1.1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -8682,17 +8678,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>BR02INP000013.1.1</t>
+          <t>BR02INP000021.1.1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>BRCPF32503272800</t>
+          <t>BRCPF09728873697</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Murilo Souza</t>
+          <t>CATHARINA SANTOS</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -8701,11 +8697,11 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>-8000</v>
+        <v>-8228.333333333332</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>R$ -8.000,00</t>
+          <t>R$ -8.228,33</t>
         </is>
       </c>
     </row>
@@ -8717,7 +8713,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>BR02CLP00161.1.1</t>
+          <t>BR02INP000013.1.1</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -8732,7 +8728,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -8752,17 +8748,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>BR02INP00002.1.2</t>
+          <t>BR02CLP00161.1.1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>BRCPF07969644910</t>
+          <t>BRCPF32503272800</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Luiz Kekis</t>
+          <t>Murilo Souza</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -8771,11 +8767,11 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>-7694.6</v>
+        <v>-8000</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>R$ -7.694,60</t>
+          <t>R$ -8.000,00</t>
         </is>
       </c>
     </row>
@@ -8787,30 +8783,30 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR02INP00002.1.2</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>BRCPF01321990685</t>
+          <t>BRCPF07969644910</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Carlos Souza</t>
+          <t>Luiz Kekis</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11, 2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>-7326.25</v>
+        <v>-7694.6</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>R$ -7.326,25</t>
+          <t>R$ -7.694,60</t>
         </is>
       </c>
     </row>
@@ -8822,30 +8818,30 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>BR02CLP00178.1.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>BRCPF03008249710</t>
+          <t>BRCPF01321990685</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Pedro Neto</t>
+          <t>Carlos Souza</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>-7140</v>
+        <v>-7326.25</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>R$ -7.140,00</t>
+          <t>R$ -7.326,25</t>
         </is>
       </c>
     </row>
@@ -8857,30 +8853,30 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>BR02INP00004.1.1</t>
+          <t>BR02CLP00178.1.1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>BRCPF39305416888</t>
+          <t>BRCPF03008249710</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Marcelo Reis</t>
+          <t>Pedro Neto</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>-6526.1</v>
+        <v>-7140</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>R$ -6.526,10</t>
+          <t>R$ -7.140,00</t>
         </is>
       </c>
     </row>
@@ -8892,17 +8888,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>BR02CLP00031.1.1</t>
+          <t>BR02INP00004.1.1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>BRCPF84585447687</t>
+          <t>BRCPF39305416888</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Silvio Jose de Souza</t>
+          <t>Marcelo Reis</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8911,11 +8907,11 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>-5830</v>
+        <v>-6526.1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>R$ -5.830,00</t>
+          <t>R$ -6.526,10</t>
         </is>
       </c>
     </row>
@@ -8927,30 +8923,30 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR02CLP00031.1.1</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>BRCPF09396903906</t>
+          <t>BRCPF84585447687</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Ronaldo Bruno De Souza Santos</t>
+          <t>Silvio Jose de Souza</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>-5826.666666666666</v>
+        <v>-5830</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>R$ -5.826,67</t>
+          <t>R$ -5.830,00</t>
         </is>
       </c>
     </row>
@@ -8962,17 +8958,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>BR02CLP00091.1.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>BRCPF36103714800</t>
+          <t>BRCPF09396903906</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Rodrigo Santos</t>
+          <t>Ronaldo Bruno De Souza Santos</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -8981,11 +8977,11 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>-5681.386666666666</v>
+        <v>-5826.666666666666</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>R$ -5.681,39</t>
+          <t>R$ -5.826,67</t>
         </is>
       </c>
     </row>
@@ -8997,30 +8993,30 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>BR02INP00004.1.1</t>
+          <t>BR02CLP00091.1.1</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>BRCPF43991981840</t>
+          <t>BRCPF36103714800</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Patricia Fernandes</t>
+          <t>Rodrigo Santos</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>-5075</v>
+        <v>-5681.386666666666</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>R$ -5.075,00</t>
+          <t>R$ -5.681,39</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9028,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>BR02INP00004.1.2</t>
+          <t>BR02INP00004.1.1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -9047,7 +9043,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -9067,30 +9063,30 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR02INP00004.1.2</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>BRCPF06908239918</t>
+          <t>BRCPF43991981840</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Ricardo Lopes</t>
+          <t>Patricia Fernandes</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>-5060</v>
+        <v>-5075</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>R$ -5.060,00</t>
+          <t>R$ -5.075,00</t>
         </is>
       </c>
     </row>
@@ -9107,25 +9103,25 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>BRCPF05779922608</t>
+          <t>BRCPF06908239918</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Danilo Dumba</t>
+          <t>Ricardo Lopes</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>-4968.425</v>
+        <v>-5060</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>R$ -4.968,43</t>
+          <t>R$ -5.060,00</t>
         </is>
       </c>
     </row>
@@ -9137,30 +9133,30 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>BR02CLP000809.1.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>BRCPF36995162889</t>
+          <t>BRCPF05779922608</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Diego Fernandes</t>
+          <t>Danilo Dumba</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11, 2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>-4830.755</v>
+        <v>-4968.425</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>R$ -4.830,76</t>
+          <t>R$ -4.968,43</t>
         </is>
       </c>
     </row>
@@ -9172,30 +9168,30 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>BR02INP000010.1.1</t>
+          <t>BR02CLP000809.1.1</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>BRCPF21248980867</t>
+          <t>BRCPF36995162889</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Samantha Garcia</t>
+          <t>Diego Fernandes</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>-4350.5</v>
+        <v>-4830.755</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>R$ -4.350,50</t>
+          <t>R$ -4.830,76</t>
         </is>
       </c>
     </row>
@@ -9237,22 +9233,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>BR07CLP00102.1.5</t>
+          <t>BR02INP000010.1.1</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>BRCPF05008651161</t>
+          <t>BRCPF21248980867</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Guilherme Laudensack</t>
+          <t>Samantha Garcia</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9261,46 +9257,46 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>-4272.390285090907</v>
+        <v>-4350.5</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>R$ -4.272,39</t>
+          <t>R$ -4.350,50</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR07CLP00102.1.5</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>BRCPF38133115892</t>
+          <t>BRCPF05008651161</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Thiago Giraldes</t>
+          <t>Guilherme Laudensack</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>-3963.508</v>
+        <v>-4272.390285090907</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>R$ -3.963,51</t>
+          <t>R$ -4.272,39</t>
         </is>
       </c>
     </row>
@@ -9312,30 +9308,30 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>BR07CLP00015.0.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>BRCPF40861701836</t>
+          <t>BRCPF38133115892</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>THIAGO RIBEIRO RETAMIRO</t>
+          <t>Thiago Giraldes</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>-3818.08</v>
+        <v>-3963.508</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>R$ -3.818,08</t>
+          <t>R$ -3.963,51</t>
         </is>
       </c>
     </row>
@@ -9347,30 +9343,30 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR07CLP00015.0.1</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>BRCPF00080118003</t>
+          <t>BRCPF40861701836</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Fabio Winck</t>
+          <t>THIAGO RIBEIRO RETAMIRO</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>-3800.08125</v>
+        <v>-3818.08</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>R$ -3.800,08</t>
+          <t>R$ -3.818,08</t>
         </is>
       </c>
     </row>
@@ -9382,30 +9378,30 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>BR02BU2020.1.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>BRCPF43642053890</t>
+          <t>BRCPF00080118003</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>MATEUS OLIVEIRA</t>
+          <t>Fabio Winck</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>-3420</v>
+        <v>-3800.08125</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>R$ -3.420,00</t>
+          <t>R$ -3.800,08</t>
         </is>
       </c>
     </row>
@@ -9417,7 +9413,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>BR02CLP000819.1.1</t>
+          <t>BR02BU2020.1.1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -9452,17 +9448,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR02CLP000819.1.1</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>BRCPF84585447687</t>
+          <t>BRCPF43642053890</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Silvio Jose de Souza</t>
+          <t>MATEUS OLIVEIRA</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -9471,11 +9467,11 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>-3410</v>
+        <v>-3420</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>R$ -3.410,00</t>
+          <t>R$ -3.420,00</t>
         </is>
       </c>
     </row>
@@ -9487,30 +9483,30 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>BR02INP000011.1.1</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>BRCPF29823044813</t>
+          <t>BRCPF84585447687</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Maria Gomes</t>
+          <t>Silvio Jose de Souza</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>-3293</v>
+        <v>-3410</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>R$ -3.293,00</t>
+          <t>R$ -3.410,00</t>
         </is>
       </c>
     </row>
@@ -9522,7 +9518,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>BR02INP000012.1.1</t>
+          <t>BR02INP000011.1.1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -9537,7 +9533,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -9557,7 +9553,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>BR02INP00004.1.1</t>
+          <t>BR02INP000013.1.1</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -9572,7 +9568,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-11, 2025-12</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -9592,7 +9588,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>BR02INP000013.1.1</t>
+          <t>BR02INP000012.1.1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -9607,7 +9603,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2025-11, 2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -9627,65 +9623,65 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>BR02CLP000115.1.1</t>
+          <t>BR02INP00004.1.1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>BRCPF01321990685</t>
+          <t>BRCPF29823044813</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Carlos Souza</t>
+          <t>Maria Gomes</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>-3006.25</v>
+        <v>-3293</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>R$ -3.006,25</t>
+          <t>R$ -3.293,00</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>BR07CLP00102.1.1</t>
+          <t>BR02CLP000115.1.1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>BRCPF33656123861</t>
+          <t>BRCPF01321990685</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Diego Grigorjevs</t>
+          <t>Carlos Souza</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2025-10, 2025-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>-2924.811818961039</v>
+        <v>-3006.25</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>R$ -2.924,81</t>
+          <t>R$ -3.006,25</t>
         </is>
       </c>
     </row>
@@ -9697,65 +9693,65 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>BR07CLP00165.1.1</t>
+          <t>BR07CLP00102.1.1</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>BRCPF41904875890-1</t>
+          <t>BRCPF33656123861</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>EMILY IZABELLE GONCALVES</t>
+          <t>Diego Grigorjevs</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-12</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>-2779.144924</v>
+        <v>-2924.811818961039</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>R$ -2.779,14</t>
+          <t>R$ -2.924,81</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>FCamara</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>BR02INP00002.1.2</t>
+          <t>BR07CLP00165.1.1</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>BRCPF33617629873</t>
+          <t>BRCPF41904875890-1</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Danielle Peraccini</t>
+          <t>EMILY IZABELLE GONCALVES</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>2025-10, 2025-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>-2700</v>
+        <v>-2779.144924</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>R$ -2.700,00</t>
+          <t>R$ -2.779,14</t>
         </is>
       </c>
     </row>
@@ -9767,30 +9763,30 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>BR02CLP00241.1.1</t>
+          <t>BR02INP00002.1.2</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>BRCPF11340898640</t>
+          <t>BRCPF33617629873</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Matheus Fraga</t>
+          <t>Danielle Peraccini</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2025-10, 2025-11</t>
+          <t>2025-10, 2025-12</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>-2300</v>
+        <v>-2700</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>R$ -2.300,00</t>
+          <t>R$ -2.700,00</t>
         </is>
       </c>
     </row>
@@ -9837,17 +9833,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>BR02INP00009.1.1</t>
+          <t>BR02CLP00241.1.1</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>BRCPF48959910678</t>
+          <t>BRCPF11340898640</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Joao Braccini</t>
+          <t>Matheus Fraga</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -9856,46 +9852,46 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>-1635.555555555555</v>
+        <v>-2300</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>R$ -1.635,56</t>
+          <t>R$ -2.300,00</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Hyper</t>
+          <t>FCamara</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>BR07CLP00180.1.4</t>
+          <t>BR02INP00009.1.1</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>BRCPF40625247833</t>
+          <t>BRCPF48959910678</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Luana Arena</t>
+          <t>Joao Braccini</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-10, 2025-11</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>-1442.829992181818</v>
+        <v>-1635.555555555555</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>R$ -1.442,83</t>
+          <t>R$ -1.635,56</t>
         </is>
       </c>
     </row>
@@ -9907,17 +9903,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>BR07CLP00102.1.5</t>
+          <t>BR07CLP00180.1.4</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>BRCPF33656123861</t>
+          <t>BRCPF40625247833</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Diego Grigorjevs</t>
+          <t>Luana Arena</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -9926,46 +9922,46 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>-1364.912182181818</v>
+        <v>-1442.829992181818</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>R$ -1.364,91</t>
+          <t>R$ -1.442,83</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>BR07</t>
+          <t>Hyper</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>BR07CLP00126.0.1</t>
+          <t>BR07CLP00102.1.5</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>BRCPF00671466780</t>
+          <t>BRCPF33656123861</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Adriana Fonseca Pinto</t>
+          <t>Diego Grigorjevs</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>-483.93</v>
+        <v>-1364.912182181818</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>R$ -483,93</t>
+          <t>R$ -1.364,91</t>
         </is>
       </c>
     </row>
@@ -9980,14 +9976,10 @@
           <t>BR07CLP00126.0.1</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>BRCPF39496114873</t>
-        </is>
-      </c>
+      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Mariana Goto da Silva</t>
+          <t>Adriana Fonseca Pinto</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -9996,33 +9988,29 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>316.6799999999998</v>
+        <v>-483.93</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>R$ 316,68</t>
+          <t>R$ -483,93</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BR02</t>
+          <t>BR07</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>BR02CLP000123.0.1</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>BRCPF23633749837</t>
-        </is>
-      </c>
+          <t>BR07CLP00006.0.1</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>EVELYN HIKARI YOSHITANI</t>
+          <t>Kaique Spagnol Tofoli</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -10031,33 +10019,29 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>727.05</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>R$ 727,05</t>
+          <t>R$ 83,10</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>BR02</t>
+          <t>BR07</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>BR02CLP000312.0.1</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>BRCPF09728873697</t>
-        </is>
-      </c>
+          <t>BR07CLP00084.0.3</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
-          <t>CATHARINA  GAISSLER SANTOS</t>
+          <t>Renan De Andrade Vedana</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -10066,33 +10050,29 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>1378.38</v>
+        <v>115.31</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>R$ 1.378,38</t>
+          <t>R$ 115,31</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>BR02</t>
+          <t>BR07</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>BR02CLP000234.0.1</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>BRCPF43991981840</t>
-        </is>
-      </c>
+          <t>BR07CLP00126.0.1</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Patricia Costa Fernandes</t>
+          <t>Mariana Goto da Silva</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -10101,11 +10081,11 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>4319.14</v>
+        <v>316.6799999999998</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>R$ 4.319,14</t>
+          <t>R$ 316,68</t>
         </is>
       </c>
     </row>
@@ -10117,28 +10097,210 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
+          <t>BR02CLP000123.0.1</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>EVELYN HIKARI YOSHITANI</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>727.05</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>R$ 727,05</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>BR09</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BR09CLP00003.0.1</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Lucas Angeli</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>956.9699999999993</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>R$ 956,97</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>BR02</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>BR02CLP000312.0.1</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>CATHARINA  GAISSLER SANTOS</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>1378.38</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>R$ 1.378,38</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>BR09</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>BR09CLP00004.0.1</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Brayan Bernardo de Souza</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>1493.73</v>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>R$ 1.493,73</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>BR09</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BR09CLP00008.0.1</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Tatiane Correa Camilo</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>1648.56</v>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>R$ 1.648,56</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>BR02</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>BR02CLP000234.0.1</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Patricia Costa Fernandes</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>4319.14</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>R$ 4.319,14</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>BR02</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
           <t>BR02CLP00115.0.1</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>BRCPF40254370829</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
         <is>
           <t>Guilherme Manucci</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
+      <c r="E140" t="inlineStr">
         <is>
           <t>2025-10, 2025-11</t>
         </is>
       </c>
-      <c r="F134" t="n">
+      <c r="F140" t="n">
         <v>33559.52</v>
       </c>
-      <c r="G134" t="inlineStr">
+      <c r="G140" t="inlineStr">
         <is>
           <t>R$ 33.559,52</t>
         </is>

</xml_diff>